<commit_message>
Atualização automática portal obras
</commit_message>
<xml_diff>
--- a/upload/coordenadas.xlsx
+++ b/upload/coordenadas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F900"/>
+  <dimension ref="A1:F920"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24970,7 +24970,11 @@
           <t>DM-9512044/2026</t>
         </is>
       </c>
-      <c r="B829" t="inlineStr"/>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>9512044</t>
+        </is>
+      </c>
       <c r="C829" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25474,7 +25478,11 @@
           <t>DC-9511902/2026</t>
         </is>
       </c>
-      <c r="B847" t="inlineStr"/>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
       <c r="C847" t="inlineStr">
         <is>
           <t>Obra 4</t>
@@ -25490,7 +25498,11 @@
           <t>DC-9511902/2026</t>
         </is>
       </c>
-      <c r="B848" t="inlineStr"/>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
       <c r="C848" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25506,7 +25518,11 @@
           <t>DC-9511902/2026</t>
         </is>
       </c>
-      <c r="B849" t="inlineStr"/>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
       <c r="C849" t="inlineStr">
         <is>
           <t>Obra 3</t>
@@ -25522,7 +25538,11 @@
           <t>DC-9511902/2026</t>
         </is>
       </c>
-      <c r="B850" t="inlineStr"/>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>9511902</t>
+        </is>
+      </c>
       <c r="C850" t="inlineStr">
         <is>
           <t>Obra 2</t>
@@ -25538,7 +25558,11 @@
           <t>DM-9519034/2026</t>
         </is>
       </c>
-      <c r="B851" t="inlineStr"/>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>9519034</t>
+        </is>
+      </c>
       <c r="C851" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25554,7 +25578,11 @@
           <t>DC-9519020/2026</t>
         </is>
       </c>
-      <c r="B852" t="inlineStr"/>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>9519020</t>
+        </is>
+      </c>
       <c r="C852" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25602,7 +25630,11 @@
           <t>DC-9519017/2026</t>
         </is>
       </c>
-      <c r="B854" t="inlineStr"/>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>9519017</t>
+        </is>
+      </c>
       <c r="C854" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25626,7 +25658,11 @@
           <t>DC-9519295/2026</t>
         </is>
       </c>
-      <c r="B855" t="inlineStr"/>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>9519295</t>
+        </is>
+      </c>
       <c r="C855" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25650,7 +25686,11 @@
           <t>DC-9519295/2026</t>
         </is>
       </c>
-      <c r="B856" t="inlineStr"/>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>9519295</t>
+        </is>
+      </c>
       <c r="C856" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25674,7 +25714,11 @@
           <t>DC-9518140/2026</t>
         </is>
       </c>
-      <c r="B857" t="inlineStr"/>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>9518140</t>
+        </is>
+      </c>
       <c r="C857" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25698,7 +25742,11 @@
           <t>DC-9518140/2026</t>
         </is>
       </c>
-      <c r="B858" t="inlineStr"/>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>9518140</t>
+        </is>
+      </c>
       <c r="C858" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25754,7 +25802,11 @@
           <t>DM-007/2024-A</t>
         </is>
       </c>
-      <c r="B860" t="inlineStr"/>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>9422060</t>
+        </is>
+      </c>
       <c r="C860" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -25854,12 +25906,12 @@
       </c>
       <c r="D863" t="inlineStr">
         <is>
-          <t>-17.03493425248546</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E863" t="inlineStr">
         <is>
-          <t>-46.58862620066699</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F863" t="inlineStr">
@@ -25886,12 +25938,12 @@
       </c>
       <c r="D864" t="inlineStr">
         <is>
-          <t>-17.03493425248546</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E864" t="inlineStr">
         <is>
-          <t>-46.58862620066699</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F864" t="inlineStr">
@@ -25913,17 +25965,17 @@
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
         <is>
-          <t>-17.21201508102213</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E865" t="inlineStr">
         <is>
-          <t>-46.687872082284</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F865" t="inlineStr">
@@ -25945,17 +25997,17 @@
       </c>
       <c r="C866" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
         <is>
-          <t>-17.21201508102213</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E866" t="inlineStr">
         <is>
-          <t>-46.687872082284</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F866" t="inlineStr">
@@ -25977,17 +26029,17 @@
       </c>
       <c r="C867" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
         <is>
-          <t>-17.10715545158923</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E867" t="inlineStr">
         <is>
-          <t>-46.62095644999281</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F867" t="inlineStr">
@@ -26009,17 +26061,17 @@
       </c>
       <c r="C868" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 2</t>
         </is>
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>-17.10715545158923</t>
+          <t>-17.03493425248546</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
         <is>
-          <t>-46.62095644999281</t>
+          <t>-46.58862620066699</t>
         </is>
       </c>
       <c r="F868" t="inlineStr">
@@ -26031,74 +26083,110 @@
     <row r="869">
       <c r="A869" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B869" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C869" t="inlineStr">
         <is>
-          <t>Obra 3</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>-21.27464910003665</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E869" t="inlineStr">
         <is>
-          <t>-42.91331545001727</t>
-        </is>
-      </c>
-      <c r="F869" t="inlineStr"/>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="870">
       <c r="A870" t="inlineStr">
         <is>
-          <t>DC-9501894/2026</t>
-        </is>
-      </c>
-      <c r="B870" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C870" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D870" t="inlineStr"/>
-      <c r="E870" t="inlineStr"/>
-      <c r="F870" t="inlineStr"/>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>-17.21201508102213</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="871">
       <c r="A871" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B871" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C871" t="inlineStr">
         <is>
-          <t>Obra 2</t>
+          <t>Obra 1</t>
         </is>
       </c>
       <c r="D871" t="inlineStr">
         <is>
-          <t>-21.23264738347681</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E871" t="inlineStr">
         <is>
-          <t>-43.43361939286979</t>
-        </is>
-      </c>
-      <c r="F871" t="inlineStr"/>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="872">
       <c r="A872" t="inlineStr">
         <is>
-          <t>DC-9515457/2026</t>
-        </is>
-      </c>
-      <c r="B872" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C872" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26106,25 +26194,29 @@
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>-21.23528484003703</t>
+          <t>-17.21201508102213</t>
         </is>
       </c>
       <c r="E872" t="inlineStr">
         <is>
-          <t>-43.44604111152106</t>
-        </is>
-      </c>
-      <c r="F872" t="inlineStr"/>
+          <t>-46.687872082284</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="873">
       <c r="A873" t="inlineStr">
         <is>
-          <t>DO-009482017/2025-L3</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>9482017</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
@@ -26134,29 +26226,29 @@
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F873" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="874">
       <c r="A874" t="inlineStr">
         <is>
-          <t>DO-9493205/2026-L4</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>9493205</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
@@ -26166,27 +26258,31 @@
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E874" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F874" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="875">
       <c r="A875" t="inlineStr">
         <is>
-          <t>DO-009482032/2025-L6</t>
-        </is>
-      </c>
-      <c r="B875" t="inlineStr"/>
+          <t>DC-9507997/2026</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>9507997</t>
+        </is>
+      </c>
       <c r="C875" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26194,25 +26290,29 @@
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E875" t="inlineStr">
         <is>
-          <t>-43.983052</t>
-        </is>
-      </c>
-      <c r="F875" t="inlineStr"/>
+          <t>-46.62095644999281</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>1301606 000002/2026</t>
+        </is>
+      </c>
     </row>
     <row r="876">
       <c r="A876" t="inlineStr">
         <is>
-          <t>DO-9481987/2025-L7</t>
+          <t>DC-9507997/2026</t>
         </is>
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>9481987</t>
+          <t>9507997</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
@@ -26222,61 +26322,57 @@
       </c>
       <c r="D876" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-17.10715545158923</t>
         </is>
       </c>
       <c r="E876" t="inlineStr">
         <is>
-          <t>-43.983052</t>
+          <t>-46.62095644999281</t>
         </is>
       </c>
       <c r="F876" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>1301606 000002/2026</t>
         </is>
       </c>
     </row>
     <row r="877">
       <c r="A877" t="inlineStr">
         <is>
-          <t>DO-009482055/2025-L5</t>
+          <t>DC-9515457/2026</t>
         </is>
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>9482055</t>
+          <t>9515457</t>
         </is>
       </c>
       <c r="C877" t="inlineStr">
         <is>
-          <t>Obra 1</t>
+          <t>Obra 3</t>
         </is>
       </c>
       <c r="D877" t="inlineStr">
         <is>
-          <t>-19.9275586</t>
+          <t>-21.27464910003665</t>
         </is>
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>-43.983052</t>
-        </is>
-      </c>
-      <c r="F877" t="inlineStr">
-        <is>
-          <t>2301901 000001/2025</t>
-        </is>
-      </c>
+          <t>-42.91331545001727</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr"/>
     </row>
     <row r="878">
       <c r="A878" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DC-9501894/2026</t>
         </is>
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9501894</t>
         </is>
       </c>
       <c r="C878" t="inlineStr">
@@ -26286,43 +26382,47 @@
       </c>
       <c r="D878" t="inlineStr"/>
       <c r="E878" t="inlineStr"/>
-      <c r="F878" t="inlineStr">
-        <is>
-          <t>2301617 000003/2025</t>
-        </is>
-      </c>
+      <c r="F878" t="inlineStr"/>
     </row>
     <row r="879">
       <c r="A879" t="inlineStr">
         <is>
-          <t>AMA-9499286/2026</t>
+          <t>DC-9515457/2026</t>
         </is>
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>9499286</t>
+          <t>9515457</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
         <is>
-          <t>Obra 1</t>
-        </is>
-      </c>
-      <c r="D879" t="inlineStr"/>
-      <c r="E879" t="inlineStr"/>
-      <c r="F879" t="inlineStr">
-        <is>
-          <t>2301617 000003/2025</t>
-        </is>
-      </c>
+          <t>Obra 2</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>-21.23264738347681</t>
+        </is>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>-43.43361939286979</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr"/>
     </row>
     <row r="880">
       <c r="A880" t="inlineStr">
         <is>
-          <t>DC-9519595/2026</t>
-        </is>
-      </c>
-      <c r="B880" t="inlineStr"/>
+          <t>DC-9515457/2026</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>9515457</t>
+        </is>
+      </c>
       <c r="C880" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26330,12 +26430,12 @@
       </c>
       <c r="D880" t="inlineStr">
         <is>
-          <t>-19.2091689</t>
+          <t>-21.23528484003703</t>
         </is>
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>-44.24819679999999</t>
+          <t>-43.44604111152106</t>
         </is>
       </c>
       <c r="F880" t="inlineStr"/>
@@ -26343,10 +26443,14 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>DC-9519595/2026</t>
-        </is>
-      </c>
-      <c r="B881" t="inlineStr"/>
+          <t>DO-009482017/2025-L3</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>9482017</t>
+        </is>
+      </c>
       <c r="C881" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26354,25 +26458,29 @@
       </c>
       <c r="D881" t="inlineStr">
         <is>
-          <t>-19.347297668442856</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>-44.17816254149293</t>
-        </is>
-      </c>
-      <c r="F881" t="inlineStr"/>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
     </row>
     <row r="882">
       <c r="A882" t="inlineStr">
         <is>
-          <t>DM-9497685/2026</t>
+          <t>DO-9493205/2026-L4</t>
         </is>
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>9497685</t>
+          <t>9493205</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
@@ -26380,23 +26488,31 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D882" t="inlineStr"/>
-      <c r="E882" t="inlineStr"/>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>-19.9275586</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>-43.983052</t>
+        </is>
+      </c>
       <c r="F882" t="inlineStr">
         <is>
-          <t>2301762 000023/2025</t>
+          <t>2301901 000001/2025</t>
         </is>
       </c>
     </row>
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>DM-005/2024-A</t>
+          <t>DO-009482032/2025-L6</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>9414460</t>
+          <t>9482032</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
@@ -26406,27 +26522,27 @@
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>-19.7469167</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>-47.9483714</t>
-        </is>
-      </c>
-      <c r="F883" t="inlineStr">
-        <is>
-          <t>2301762 000036/2023</t>
-        </is>
-      </c>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr"/>
     </row>
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>DC-9518766/2026</t>
-        </is>
-      </c>
-      <c r="B884" t="inlineStr"/>
+          <t>DO-9481987/2025-L7</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>9481987</t>
+        </is>
+      </c>
       <c r="C884" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26434,23 +26550,31 @@
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>-15.483562</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E884" t="inlineStr">
         <is>
-          <t>-44.39677500000001</t>
-        </is>
-      </c>
-      <c r="F884" t="inlineStr"/>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>DC-9518766/2026</t>
-        </is>
-      </c>
-      <c r="B885" t="inlineStr"/>
+          <t>DO-009482055/2025-L5</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>9482055</t>
+        </is>
+      </c>
       <c r="C885" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26458,23 +26582,31 @@
       </c>
       <c r="D885" t="inlineStr">
         <is>
-          <t>-15.5007309</t>
+          <t>-19.9275586</t>
         </is>
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>-44.7624674</t>
-        </is>
-      </c>
-      <c r="F885" t="inlineStr"/>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
     </row>
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>DM-9500304/2026</t>
-        </is>
-      </c>
-      <c r="B886" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C886" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26482,63 +26614,71 @@
       </c>
       <c r="D886" t="inlineStr"/>
       <c r="E886" t="inlineStr"/>
-      <c r="F886" t="inlineStr"/>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>DC-9519740/2026</t>
-        </is>
-      </c>
-      <c r="B887" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C887" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D887" t="inlineStr">
-        <is>
-          <t>-22.087663382295393</t>
-        </is>
-      </c>
-      <c r="E887" t="inlineStr">
-        <is>
-          <t>-46.558100143637475</t>
-        </is>
-      </c>
-      <c r="F887" t="inlineStr"/>
+      <c r="D887" t="inlineStr"/>
+      <c r="E887" t="inlineStr"/>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>DC-9519740/2026</t>
-        </is>
-      </c>
-      <c r="B888" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C888" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D888" t="inlineStr">
-        <is>
-          <t>-22.047693352827803</t>
-        </is>
-      </c>
-      <c r="E888" t="inlineStr">
-        <is>
-          <t>-46.555137035221186</t>
-        </is>
-      </c>
-      <c r="F888" t="inlineStr"/>
+      <c r="D888" t="inlineStr"/>
+      <c r="E888" t="inlineStr"/>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AMA-9502187/2026</t>
-        </is>
-      </c>
-      <c r="B889" t="inlineStr"/>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
       <c r="C889" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26546,7 +26686,11 @@
       </c>
       <c r="D889" t="inlineStr"/>
       <c r="E889" t="inlineStr"/>
-      <c r="F889" t="inlineStr"/>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
@@ -26599,12 +26743,12 @@
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>DO-009482046/2025-L2</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>9482046</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
@@ -26612,31 +26756,23 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D892" t="inlineStr">
-        <is>
-          <t>-19.9275586</t>
-        </is>
-      </c>
-      <c r="E892" t="inlineStr">
-        <is>
-          <t>-43.983052</t>
-        </is>
-      </c>
+      <c r="D892" t="inlineStr"/>
+      <c r="E892" t="inlineStr"/>
       <c r="F892" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
-          <t>DO-009482014/2025-L1</t>
+          <t>AMA-9499286/2026</t>
         </is>
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>9482014</t>
+          <t>9499286</t>
         </is>
       </c>
       <c r="C893" t="inlineStr">
@@ -26644,29 +26780,25 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D893" t="inlineStr">
-        <is>
-          <t>-19.9275586</t>
-        </is>
-      </c>
-      <c r="E893" t="inlineStr">
-        <is>
-          <t>-43.983052</t>
-        </is>
-      </c>
+      <c r="D893" t="inlineStr"/>
+      <c r="E893" t="inlineStr"/>
       <c r="F893" t="inlineStr">
         <is>
-          <t>2301901 000001/2025</t>
+          <t>2301617 000003/2025</t>
         </is>
       </c>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
         <is>
-          <t>DM-9512043/2026</t>
-        </is>
-      </c>
-      <c r="B894" t="inlineStr"/>
+          <t>DC-9519595/2026</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>9519295</t>
+        </is>
+      </c>
       <c r="C894" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26674,12 +26806,12 @@
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>-16.7203311</t>
+          <t>-19.2091689</t>
         </is>
       </c>
       <c r="E894" t="inlineStr">
         <is>
-          <t>-43.8541147</t>
+          <t>-44.24819679999999</t>
         </is>
       </c>
       <c r="F894" t="inlineStr"/>
@@ -26687,10 +26819,14 @@
     <row r="895">
       <c r="A895" t="inlineStr">
         <is>
-          <t>DC-9518942/2026</t>
-        </is>
-      </c>
-      <c r="B895" t="inlineStr"/>
+          <t>DC-9519595/2026</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>9519295</t>
+        </is>
+      </c>
       <c r="C895" t="inlineStr">
         <is>
           <t>Obra 1</t>
@@ -26698,12 +26834,12 @@
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>-16.964100809511475</t>
+          <t>-19.347297668442856</t>
         </is>
       </c>
       <c r="E895" t="inlineStr">
         <is>
-          <t>-46.40676935458991</t>
+          <t>-44.17816254149293</t>
         </is>
       </c>
       <c r="F895" t="inlineStr"/>
@@ -26711,36 +26847,36 @@
     <row r="896">
       <c r="A896" t="inlineStr">
         <is>
-          <t>DC-9518942/2026</t>
-        </is>
-      </c>
-      <c r="B896" t="inlineStr"/>
+          <t>DM-9497685/2026</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>9497685</t>
+        </is>
+      </c>
       <c r="C896" t="inlineStr">
         <is>
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D896" t="inlineStr">
-        <is>
-          <t>-16.985130778257258</t>
-        </is>
-      </c>
-      <c r="E896" t="inlineStr">
-        <is>
-          <t>-46.27544298436485</t>
-        </is>
-      </c>
-      <c r="F896" t="inlineStr"/>
+      <c r="D896" t="inlineStr"/>
+      <c r="E896" t="inlineStr"/>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>2301762 000023/2025</t>
+        </is>
+      </c>
     </row>
     <row r="897">
       <c r="A897" t="inlineStr">
         <is>
-          <t>DM-011/2024-A</t>
+          <t>DM-005/2024-A</t>
         </is>
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>9421657</t>
+          <t>9414460</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
@@ -26750,12 +26886,12 @@
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>-17.335013</t>
+          <t>-19.7469167</t>
         </is>
       </c>
       <c r="E897" t="inlineStr">
         <is>
-          <t>-44.943418</t>
+          <t>-47.9483714</t>
         </is>
       </c>
       <c r="F897" t="inlineStr">
@@ -26767,12 +26903,12 @@
     <row r="898">
       <c r="A898" t="inlineStr">
         <is>
-          <t>DM-010/2024-A</t>
+          <t>DC-9518766/2026</t>
         </is>
       </c>
       <c r="B898" t="inlineStr">
         <is>
-          <t>9418600</t>
+          <t>9518766</t>
         </is>
       </c>
       <c r="C898" t="inlineStr">
@@ -26780,23 +26916,27 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D898" t="inlineStr"/>
-      <c r="E898" t="inlineStr"/>
-      <c r="F898" t="inlineStr">
-        <is>
-          <t>2301762 000036/2023</t>
-        </is>
-      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>-15.483562</t>
+        </is>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>-44.39677500000001</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr"/>
     </row>
     <row r="899">
       <c r="A899" t="inlineStr">
         <is>
-          <t>DM-009/2024-A</t>
+          <t>DC-9518766/2026</t>
         </is>
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>9422078</t>
+          <t>9518766</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
@@ -26804,23 +26944,27 @@
           <t>Obra 1</t>
         </is>
       </c>
-      <c r="D899" t="inlineStr"/>
-      <c r="E899" t="inlineStr"/>
-      <c r="F899" t="inlineStr">
-        <is>
-          <t>2301762 000036/2023</t>
-        </is>
-      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>-15.5007309</t>
+        </is>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>-44.7624674</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr"/>
     </row>
     <row r="900">
       <c r="A900" t="inlineStr">
         <is>
-          <t>DM-008/2024-A</t>
+          <t>DM-9500304/2026</t>
         </is>
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>9422064</t>
+          <t>9500304</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
@@ -26830,7 +26974,519 @@
       </c>
       <c r="D900" t="inlineStr"/>
       <c r="E900" t="inlineStr"/>
-      <c r="F900" t="inlineStr">
+      <c r="F900" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>DC-9519740/2026</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>9519740</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>-22.087663382295393</t>
+        </is>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>-46.558100143637475</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>DC-9519740/2026</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>9519740</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>-22.047693352827803</t>
+        </is>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>-46.555137035221186</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AMA-9502187/2026</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr"/>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr"/>
+      <c r="E903" t="inlineStr"/>
+      <c r="F903" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr"/>
+      <c r="E904" t="inlineStr"/>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr"/>
+      <c r="E905" t="inlineStr"/>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr"/>
+      <c r="E906" t="inlineStr"/>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr"/>
+      <c r="E907" t="inlineStr"/>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr"/>
+      <c r="E908" t="inlineStr"/>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr"/>
+      <c r="E909" t="inlineStr"/>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr"/>
+      <c r="E910" t="inlineStr"/>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>AMA-9499286/2026</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>9499286</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr"/>
+      <c r="E911" t="inlineStr"/>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>2301617 000003/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>DO-009482046/2025-L2</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>9482046</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>-19.9275586</t>
+        </is>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>DO-009482014/2025-L1</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>9482014</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>-19.9275586</t>
+        </is>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>-43.983052</t>
+        </is>
+      </c>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>2301901 000001/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>DM-9512043/2026</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>9512043</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>-16.7203311</t>
+        </is>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>-43.8541147</t>
+        </is>
+      </c>
+      <c r="F914" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>DC-9518942/2026</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>9518942</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>-16.964100809511475</t>
+        </is>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>-46.40676935458991</t>
+        </is>
+      </c>
+      <c r="F915" t="inlineStr"/>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>DC-9518942/2026</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>9518942</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>-16.985130778257258</t>
+        </is>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>-46.27544298436485</t>
+        </is>
+      </c>
+      <c r="F916" t="inlineStr"/>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>DM-011/2024-A</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>9421657</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>-17.335013</t>
+        </is>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>-44.943418</t>
+        </is>
+      </c>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>2301762 000036/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>DM-010/2024-A</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>9418600</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr"/>
+      <c r="E918" t="inlineStr"/>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>2301762 000036/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>DM-009/2024-A</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>9422078</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr"/>
+      <c r="E919" t="inlineStr"/>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>2301762 000036/2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>DM-008/2024-A</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>9422064</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>Obra 1</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr"/>
+      <c r="E920" t="inlineStr"/>
+      <c r="F920" t="inlineStr">
         <is>
           <t>2301762 000036/2023</t>
         </is>

</xml_diff>